<commit_message>
completed Entire Project(Completed Expense.jsx, Income.jsx, TimeFrame.jsx, index.css, TransactionItem.jsx, exportUtiljsx, Profile.jsx)
</commit_message>
<xml_diff>
--- a/Backend/expense_details.xlsx
+++ b/Backend/expense_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,35 +415,91 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Fast food</v>
+        <v>Groceries</v>
       </c>
       <c r="B2">
-        <v>1000</v>
+        <v>105</v>
       </c>
       <c r="C2" t="str">
-        <v>food</v>
+        <v>Food</v>
       </c>
       <c r="D2" t="str">
-        <v>4/9/2026</v>
+        <v>5/12/2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Office Supplies</v>
+      </c>
+      <c r="B3">
+        <v>150.5</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Shopping</v>
+      </c>
+      <c r="D3" t="str">
+        <v>5/12/2026</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Protein Powder</v>
+      </c>
+      <c r="B4">
+        <v>1000</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Food</v>
+      </c>
+      <c r="D4" t="str">
+        <v>5/11/2026</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Shirt</v>
+      </c>
+      <c r="B5">
+        <v>163</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Shopping</v>
+      </c>
+      <c r="D5" t="str">
+        <v>5/11/2026</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Fast food</v>
+      </c>
+      <c r="B6">
+        <v>1000</v>
+      </c>
+      <c r="C6" t="str">
+        <v>food</v>
+      </c>
+      <c r="D6" t="str">
+        <v>4/9/2026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>Snacks</v>
       </c>
-      <c r="B3">
+      <c r="B7">
         <v>900</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C7" t="str">
         <v>food</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D7" t="str">
         <v>4/9/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>